<commit_message>
Build AI Action Centre workflow
</commit_message>
<xml_diff>
--- a/ev_lifecycle_template.xlsx
+++ b/ev_lifecycle_template.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -841,7 +841,7 @@
     <row r="26" ht="20" customHeight="1">
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>currentKm</t>
+          <t>warrantyExpiryDate</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -851,19 +851,19 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Positive integer (e.g. 1500)</t>
+          <t>YYYY-MM-DD (Date)</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>Current odometer reading in kilometers (Defaults to 0).</t>
+          <t>Vehicle warranty expiry date used by lifecycle risk rules.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>registrationStatus</t>
+          <t>lastCustomerContactDate</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
@@ -873,19 +873,19 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>delivered / documents_pending / submitted / completed</t>
+          <t>YYYY-MM-DD (Date)</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>Current status of RTO registration.</t>
+          <t>Date of the most recent customer contact attempt.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>registrationNumber</t>
+          <t>lastCustomerContactOutcome</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
@@ -895,19 +895,19 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Registration plate string (e.g. MH-02-XX-1234)</t>
+          <t>connected / no_answer / message_sent</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>Assigned RTO vehicle registration plate number.</t>
+          <t>Outcome of the most recent customer contact.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>batteryReplacementAffected</t>
+          <t>issueCode</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -917,19 +917,19 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>TRUE / FALSE</t>
+          <t>Short issue code</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>Whether vehicle is part of a battery replacement campaign.</t>
+          <t>Active battery or service issue code used for pattern detection.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>batteryReplacementCampaignId</t>
+          <t>issueReportedDate</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
@@ -939,19 +939,19 @@
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Alphanumeric string (e.g. BC-2024-001)</t>
+          <t>YYYY-MM-DD (Date)</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Recall or upgrade campaign reference ID.</t>
+          <t>Date the active issue was first reported.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>batteryReplacementStatus</t>
+          <t>currentKm</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
@@ -961,19 +961,19 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>not_affected / pending / in_progress / completed</t>
+          <t>Positive integer (e.g. 1500)</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>Upgrade campaign implementation status.</t>
+          <t>Current odometer reading in kilometers (Defaults to 0).</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>batteryReplacementOldSerial</t>
+          <t>registrationStatus</t>
         </is>
       </c>
       <c r="C32" s="13" t="inlineStr">
@@ -983,19 +983,19 @@
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Alphanumeric string</t>
+          <t>delivered / documents_pending / submitted / completed</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>Serial number of the decommissioned battery.</t>
+          <t>Current status of RTO registration.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>batteryReplacementNewSerial</t>
+          <t>registrationNumber</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -1005,19 +1005,19 @@
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Alphanumeric string</t>
+          <t>Registration plate string (e.g. MH-02-XX-1234)</t>
         </is>
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>Serial number of the newly fitted battery pack.</t>
+          <t>Assigned RTO vehicle registration plate number.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>batteryReplacementDate</t>
+          <t>batteryReplacementAffected</t>
         </is>
       </c>
       <c r="C34" s="13" t="inlineStr">
@@ -1027,19 +1027,19 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD (Date)</t>
+          <t>TRUE / FALSE</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>Date of battery service upgrade completion.</t>
+          <t>Whether vehicle is part of a battery replacement campaign.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>batteryReplacementTechnician</t>
+          <t>batteryReplacementCampaignId</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
@@ -1049,32 +1049,142 @@
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Technician Name string</t>
+          <t>Alphanumeric string (e.g. BC-2024-001)</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>Technician who carried out the replacement.</t>
+          <t>Recall or upgrade campaign reference ID.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="B36" s="6" t="inlineStr">
         <is>
+          <t>batteryReplacementStatus</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>not_affected / pending / in_progress / completed</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade campaign implementation status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>batteryReplacementOldSerial</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>Alphanumeric string</t>
+        </is>
+      </c>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>Serial number of the decommissioned battery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>batteryReplacementNewSerial</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Alphanumeric string</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Serial number of the newly fitted battery pack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>batteryReplacementDate</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD (Date)</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Date of battery service upgrade completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>batteryReplacementTechnician</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Technician Name string</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Technician who carried out the replacement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="B41" s="9" t="inlineStr">
+        <is>
           <t>batteryReplacementCustomerConfirmed</t>
         </is>
       </c>
-      <c r="C36" s="13" t="inlineStr">
+      <c r="C41" s="12" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="D41" s="11" t="inlineStr">
         <is>
           <t>TRUE / FALSE</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E41" s="11" t="inlineStr">
         <is>
           <t>Customer signed-off/confirmed the upgrade.</t>
         </is>
@@ -1091,7 +1201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:Z19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1100,21 +1210,26 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="32" customWidth="1" min="15" max="15"/>
-    <col width="28" customWidth="1" min="16" max="16"/>
-    <col width="31" customWidth="1" min="17" max="17"/>
-    <col width="31" customWidth="1" min="18" max="18"/>
-    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
     <col width="32" customWidth="1" min="20" max="20"/>
-    <col width="39" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
+    <col width="31" customWidth="1" min="22" max="22"/>
+    <col width="31" customWidth="1" min="23" max="23"/>
+    <col width="26" customWidth="1" min="24" max="24"/>
+    <col width="32" customWidth="1" min="25" max="25"/>
+    <col width="39" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1170,55 +1285,80 @@
       </c>
       <c r="K1" s="5" t="inlineStr">
         <is>
+          <t>warrantyExpiryDate</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>lastCustomerContactDate</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>lastCustomerContactOutcome</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>issueCode</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>issueReportedDate</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
           <t>currentKm</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>registrationStatus</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="R1" s="5" t="inlineStr">
         <is>
           <t>registrationNumber</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="S1" s="5" t="inlineStr">
         <is>
           <t>batteryReplacementAffected</t>
         </is>
       </c>
-      <c r="O1" s="5" t="inlineStr">
+      <c r="T1" s="5" t="inlineStr">
         <is>
           <t>batteryReplacementCampaignId</t>
         </is>
       </c>
-      <c r="P1" s="5" t="inlineStr">
+      <c r="U1" s="5" t="inlineStr">
         <is>
           <t>batteryReplacementStatus</t>
         </is>
       </c>
-      <c r="Q1" s="5" t="inlineStr">
+      <c r="V1" s="5" t="inlineStr">
         <is>
           <t>batteryReplacementOldSerial</t>
         </is>
       </c>
-      <c r="R1" s="5" t="inlineStr">
+      <c r="W1" s="5" t="inlineStr">
         <is>
           <t>batteryReplacementNewSerial</t>
         </is>
       </c>
-      <c r="S1" s="5" t="inlineStr">
+      <c r="X1" s="5" t="inlineStr">
         <is>
           <t>batteryReplacementDate</t>
         </is>
       </c>
-      <c r="T1" s="5" t="inlineStr">
+      <c r="Y1" s="5" t="inlineStr">
         <is>
           <t>batteryReplacementTechnician</t>
         </is>
       </c>
-      <c r="U1" s="5" t="inlineStr">
+      <c r="Z1" s="5" t="inlineStr">
         <is>
           <t>batteryReplacementCustomerConfirmed</t>
         </is>
@@ -1257,7 +1397,7 @@
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>Ananya Bose</t>
+          <t>Shaurya Sharma</t>
         </is>
       </c>
       <c r="H2" s="14" t="inlineStr">
@@ -1267,7 +1407,7 @@
       </c>
       <c r="I2" s="14" t="inlineStr">
         <is>
-          <t>Mumbai, MH</t>
+          <t>Ahmedabad, GJ</t>
         </is>
       </c>
       <c r="J2" s="14" t="inlineStr">
@@ -1275,47 +1415,72 @@
           <t>2025-11-21</t>
         </is>
       </c>
-      <c r="K2" s="14" t="n">
-        <v>7713</v>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>2027-11-21</t>
+        </is>
       </c>
       <c r="L2" s="14" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="M2" s="14" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="N2" s="14" t="inlineStr">
+        <is>
+          <t>BMS_CELL_IMBALANCE</t>
+        </is>
+      </c>
+      <c r="O2" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="P2" s="14" t="n">
+        <v>6246</v>
+      </c>
+      <c r="Q2" s="14" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M2" s="14" t="inlineStr">
-        <is>
-          <t>MH-02-LH-1058</t>
-        </is>
-      </c>
-      <c r="N2" s="14" t="inlineStr">
+      <c r="R2" s="14" t="inlineStr">
+        <is>
+          <t>GJ-01-AU-5291</t>
+        </is>
+      </c>
+      <c r="S2" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="O2" s="14" t="inlineStr">
+      <c r="T2" s="14" t="inlineStr">
         <is>
           <t>BC-2024-001</t>
         </is>
       </c>
-      <c r="P2" s="14" t="inlineStr">
+      <c r="U2" s="14" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="Q2" s="14" t="inlineStr">
+      <c r="V2" s="14" t="inlineStr">
         <is>
           <t>BP-LFP-96001</t>
         </is>
       </c>
-      <c r="R2" s="14" t="inlineStr"/>
-      <c r="S2" s="14" t="inlineStr"/>
-      <c r="T2" s="14" t="inlineStr">
-        <is>
-          <t>Sanjay Verma</t>
-        </is>
-      </c>
-      <c r="U2" s="14" t="inlineStr">
+      <c r="W2" s="14" t="inlineStr"/>
+      <c r="X2" s="14" t="inlineStr"/>
+      <c r="Y2" s="14" t="inlineStr">
+        <is>
+          <t>Manoj Sharma</t>
+        </is>
+      </c>
+      <c r="Z2" s="14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1349,12 +1514,12 @@
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2023-01-20</t>
         </is>
       </c>
       <c r="G3" s="15" t="inlineStr">
         <is>
-          <t>Kavita Joshi</t>
+          <t>Amit Sen</t>
         </is>
       </c>
       <c r="H3" s="15" t="inlineStr">
@@ -1364,51 +1529,68 @@
       </c>
       <c r="I3" s="15" t="inlineStr">
         <is>
-          <t>Mumbai, MH</t>
+          <t>Kolkata, WB</t>
         </is>
       </c>
       <c r="J3" s="15" t="inlineStr">
         <is>
-          <t>2026-02-21</t>
-        </is>
-      </c>
-      <c r="K3" s="15" t="n">
-        <v>7044</v>
+          <t>2023-01-28</t>
+        </is>
+      </c>
+      <c r="K3" s="15" t="inlineStr">
+        <is>
+          <t>2025-01-27</t>
+        </is>
       </c>
       <c r="L3" s="15" t="inlineStr">
         <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="M3" s="15" t="inlineStr">
+        <is>
+          <t>message_sent</t>
+        </is>
+      </c>
+      <c r="N3" s="15" t="inlineStr"/>
+      <c r="O3" s="15" t="inlineStr"/>
+      <c r="P3" s="15" t="n">
+        <v>32336</v>
+      </c>
+      <c r="Q3" s="15" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M3" s="15" t="inlineStr">
-        <is>
-          <t>MH-02-YR-3442</t>
-        </is>
-      </c>
-      <c r="N3" s="15" t="inlineStr">
+      <c r="R3" s="15" t="inlineStr">
+        <is>
+          <t>WB-02-JO-8041</t>
+        </is>
+      </c>
+      <c r="S3" s="15" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="O3" s="15" t="inlineStr">
+      <c r="T3" s="15" t="inlineStr">
         <is>
           <t>BC-2024-001</t>
         </is>
       </c>
-      <c r="P3" s="15" t="inlineStr">
+      <c r="U3" s="15" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="Q3" s="15" t="inlineStr">
+      <c r="V3" s="15" t="inlineStr">
         <is>
           <t>BP-NMC-72002</t>
         </is>
       </c>
-      <c r="R3" s="15" t="inlineStr"/>
-      <c r="S3" s="15" t="inlineStr"/>
-      <c r="T3" s="15" t="inlineStr"/>
-      <c r="U3" s="15" t="inlineStr">
+      <c r="W3" s="15" t="inlineStr"/>
+      <c r="X3" s="15" t="inlineStr"/>
+      <c r="Y3" s="15" t="inlineStr"/>
+      <c r="Z3" s="15" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1442,12 +1624,12 @@
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>2025-05-30</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>Pihu Chatterjee</t>
+          <t>Aarav Grover</t>
         </is>
       </c>
       <c r="H4" s="14" t="inlineStr">
@@ -1457,44 +1639,69 @@
       </c>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>Hyderabad, TS</t>
+          <t>Pune, MH</t>
         </is>
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>2025-06-08</t>
-        </is>
-      </c>
-      <c r="K4" s="14" t="n">
-        <v>8988</v>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>2028-03-09</t>
+        </is>
       </c>
       <c r="L4" s="14" t="inlineStr">
         <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="inlineStr">
+        <is>
+          <t>message_sent</t>
+        </is>
+      </c>
+      <c r="N4" s="14" t="inlineStr">
+        <is>
+          <t>BMS_CELL_IMBALANCE</t>
+        </is>
+      </c>
+      <c r="O4" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="P4" s="14" t="n">
+        <v>3790</v>
+      </c>
+      <c r="Q4" s="14" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M4" s="14" t="inlineStr">
-        <is>
-          <t>TS-09-YZ-1653</t>
-        </is>
-      </c>
-      <c r="N4" s="14" t="inlineStr">
+      <c r="R4" s="14" t="inlineStr">
+        <is>
+          <t>MH-12-VW-1406</t>
+        </is>
+      </c>
+      <c r="S4" s="14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="O4" s="14" t="inlineStr"/>
-      <c r="P4" s="14" t="inlineStr">
-        <is>
-          <t>not_affected</t>
-        </is>
-      </c>
-      <c r="Q4" s="14" t="inlineStr"/>
-      <c r="R4" s="14" t="inlineStr"/>
-      <c r="S4" s="14" t="inlineStr"/>
       <c r="T4" s="14" t="inlineStr"/>
       <c r="U4" s="14" t="inlineStr">
         <is>
+          <t>not_affected</t>
+        </is>
+      </c>
+      <c r="V4" s="14" t="inlineStr"/>
+      <c r="W4" s="14" t="inlineStr"/>
+      <c r="X4" s="14" t="inlineStr"/>
+      <c r="Y4" s="14" t="inlineStr"/>
+      <c r="Z4" s="14" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
@@ -1527,12 +1734,12 @@
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>2024-12-25</t>
+          <t>2025-04-23</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>Sunita Singh</t>
+          <t>Amit Dutta</t>
         </is>
       </c>
       <c r="H5" s="15" t="inlineStr">
@@ -1542,44 +1749,61 @@
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
-          <t>Lucknow, UP</t>
+          <t>Ahmedabad, GJ</t>
         </is>
       </c>
       <c r="J5" s="15" t="inlineStr">
         <is>
-          <t>2025-01-16</t>
-        </is>
-      </c>
-      <c r="K5" s="15" t="n">
-        <v>19304</v>
+          <t>2025-05-05</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="inlineStr">
+        <is>
+          <t>2027-05-05</t>
+        </is>
       </c>
       <c r="L5" s="15" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="M5" s="15" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="N5" s="15" t="inlineStr"/>
+      <c r="O5" s="15" t="inlineStr"/>
+      <c r="P5" s="15" t="n">
+        <v>11360</v>
+      </c>
+      <c r="Q5" s="15" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M5" s="15" t="inlineStr">
-        <is>
-          <t>UP-32-WZ-3900</t>
-        </is>
-      </c>
-      <c r="N5" s="15" t="inlineStr">
+      <c r="R5" s="15" t="inlineStr">
+        <is>
+          <t>GJ-01-MF-8541</t>
+        </is>
+      </c>
+      <c r="S5" s="15" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="O5" s="15" t="inlineStr"/>
-      <c r="P5" s="15" t="inlineStr">
-        <is>
-          <t>not_affected</t>
-        </is>
-      </c>
-      <c r="Q5" s="15" t="inlineStr"/>
-      <c r="R5" s="15" t="inlineStr"/>
-      <c r="S5" s="15" t="inlineStr"/>
       <c r="T5" s="15" t="inlineStr"/>
       <c r="U5" s="15" t="inlineStr">
         <is>
+          <t>not_affected</t>
+        </is>
+      </c>
+      <c r="V5" s="15" t="inlineStr"/>
+      <c r="W5" s="15" t="inlineStr"/>
+      <c r="X5" s="15" t="inlineStr"/>
+      <c r="Y5" s="15" t="inlineStr"/>
+      <c r="Z5" s="15" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
@@ -1612,12 +1836,12 @@
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>2023-08-10</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
-          <t>Arjun Nair</t>
+          <t>Karan Kumar</t>
         </is>
       </c>
       <c r="H6" s="14" t="inlineStr">
@@ -1627,44 +1851,61 @@
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
-          <t>Jaipur, RJ</t>
+          <t>Ahmedabad, GJ</t>
         </is>
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>2023-08-27</t>
-        </is>
-      </c>
-      <c r="K6" s="14" t="n">
-        <v>23004</v>
+          <t>2024-07-31</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
       </c>
       <c r="L6" s="14" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="M6" s="14" t="inlineStr">
+        <is>
+          <t>no_answer</t>
+        </is>
+      </c>
+      <c r="N6" s="14" t="inlineStr"/>
+      <c r="O6" s="14" t="inlineStr"/>
+      <c r="P6" s="14" t="n">
+        <v>28025</v>
+      </c>
+      <c r="Q6" s="14" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M6" s="14" t="inlineStr">
-        <is>
-          <t>RJ-14-VL-6000</t>
-        </is>
-      </c>
-      <c r="N6" s="14" t="inlineStr">
+      <c r="R6" s="14" t="inlineStr">
+        <is>
+          <t>GJ-01-YC-5279</t>
+        </is>
+      </c>
+      <c r="S6" s="14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="O6" s="14" t="inlineStr"/>
-      <c r="P6" s="14" t="inlineStr">
-        <is>
-          <t>not_affected</t>
-        </is>
-      </c>
-      <c r="Q6" s="14" t="inlineStr"/>
-      <c r="R6" s="14" t="inlineStr"/>
-      <c r="S6" s="14" t="inlineStr"/>
       <c r="T6" s="14" t="inlineStr"/>
       <c r="U6" s="14" t="inlineStr">
         <is>
+          <t>not_affected</t>
+        </is>
+      </c>
+      <c r="V6" s="14" t="inlineStr"/>
+      <c r="W6" s="14" t="inlineStr"/>
+      <c r="X6" s="14" t="inlineStr"/>
+      <c r="Y6" s="14" t="inlineStr"/>
+      <c r="Z6" s="14" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
@@ -1697,12 +1938,12 @@
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2025-11-13</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>Priya Kulkarni</t>
+          <t>Amit Jha</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
@@ -1712,51 +1953,68 @@
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>Chennai, TN</t>
+          <t>Hyderabad, TS</t>
         </is>
       </c>
       <c r="J7" s="15" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
-        </is>
-      </c>
-      <c r="K7" s="15" t="n">
-        <v>10341</v>
+          <t>2025-11-21</t>
+        </is>
+      </c>
+      <c r="K7" s="15" t="inlineStr">
+        <is>
+          <t>2027-11-21</t>
+        </is>
       </c>
       <c r="L7" s="15" t="inlineStr">
         <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="M7" s="15" t="inlineStr">
+        <is>
+          <t>message_sent</t>
+        </is>
+      </c>
+      <c r="N7" s="15" t="inlineStr"/>
+      <c r="O7" s="15" t="inlineStr"/>
+      <c r="P7" s="15" t="n">
+        <v>7146</v>
+      </c>
+      <c r="Q7" s="15" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M7" s="15" t="inlineStr">
-        <is>
-          <t>TN-09-WG-5349</t>
-        </is>
-      </c>
-      <c r="N7" s="15" t="inlineStr">
+      <c r="R7" s="15" t="inlineStr">
+        <is>
+          <t>TS-09-LN-9821</t>
+        </is>
+      </c>
+      <c r="S7" s="15" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="O7" s="15" t="inlineStr">
+      <c r="T7" s="15" t="inlineStr">
         <is>
           <t>BC-2024-001</t>
         </is>
       </c>
-      <c r="P7" s="15" t="inlineStr">
+      <c r="U7" s="15" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="Q7" s="15" t="inlineStr">
+      <c r="V7" s="15" t="inlineStr">
         <is>
           <t>BP-LFP-96006</t>
         </is>
       </c>
-      <c r="R7" s="15" t="inlineStr"/>
-      <c r="S7" s="15" t="inlineStr"/>
-      <c r="T7" s="15" t="inlineStr"/>
-      <c r="U7" s="15" t="inlineStr">
+      <c r="W7" s="15" t="inlineStr"/>
+      <c r="X7" s="15" t="inlineStr"/>
+      <c r="Y7" s="15" t="inlineStr"/>
+      <c r="Z7" s="15" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1790,12 +2048,12 @@
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
-          <t>2025-11-13</t>
+          <t>2024-11-07</t>
         </is>
       </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
-          <t>Aditya Deshmukh</t>
+          <t>Manoj Patil</t>
         </is>
       </c>
       <c r="H8" s="14" t="inlineStr">
@@ -1805,44 +2063,61 @@
       </c>
       <c r="I8" s="14" t="inlineStr">
         <is>
-          <t>Lucknow, UP</t>
+          <t>Hyderabad, TS</t>
         </is>
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
-        </is>
-      </c>
-      <c r="K8" s="14" t="n">
-        <v>8946</v>
+          <t>2024-12-01</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
       </c>
       <c r="L8" s="14" t="inlineStr">
         <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M8" s="14" t="inlineStr">
+        <is>
+          <t>message_sent</t>
+        </is>
+      </c>
+      <c r="N8" s="14" t="inlineStr"/>
+      <c r="O8" s="14" t="inlineStr"/>
+      <c r="P8" s="14" t="n">
+        <v>15267</v>
+      </c>
+      <c r="Q8" s="14" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M8" s="14" t="inlineStr">
-        <is>
-          <t>UP-32-BL-9518</t>
-        </is>
-      </c>
-      <c r="N8" s="14" t="inlineStr">
+      <c r="R8" s="14" t="inlineStr">
+        <is>
+          <t>TS-09-RI-5844</t>
+        </is>
+      </c>
+      <c r="S8" s="14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="O8" s="14" t="inlineStr"/>
-      <c r="P8" s="14" t="inlineStr">
-        <is>
-          <t>not_affected</t>
-        </is>
-      </c>
-      <c r="Q8" s="14" t="inlineStr"/>
-      <c r="R8" s="14" t="inlineStr"/>
-      <c r="S8" s="14" t="inlineStr"/>
       <c r="T8" s="14" t="inlineStr"/>
       <c r="U8" s="14" t="inlineStr">
         <is>
+          <t>not_affected</t>
+        </is>
+      </c>
+      <c r="V8" s="14" t="inlineStr"/>
+      <c r="W8" s="14" t="inlineStr"/>
+      <c r="X8" s="14" t="inlineStr"/>
+      <c r="Y8" s="14" t="inlineStr"/>
+      <c r="Z8" s="14" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
@@ -1875,12 +2150,12 @@
       </c>
       <c r="F9" s="15" t="inlineStr">
         <is>
-          <t>2025-06-02</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>Diya Pillai</t>
+          <t>Aryan Patil</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
@@ -1890,44 +2165,57 @@
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>Lucknow, UP</t>
+          <t>Mumbai, MH</t>
         </is>
       </c>
       <c r="J9" s="15" t="inlineStr">
         <is>
-          <t>2025-06-09</t>
-        </is>
-      </c>
-      <c r="K9" s="15" t="n">
-        <v>13132</v>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="K9" s="15" t="inlineStr">
+        <is>
+          <t>2028-07-06</t>
+        </is>
       </c>
       <c r="L9" s="15" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="M9" s="15" t="inlineStr">
         <is>
-          <t>UP-32-WS-5920</t>
-        </is>
-      </c>
-      <c r="N9" s="15" t="inlineStr">
+          <t>no_answer</t>
+        </is>
+      </c>
+      <c r="N9" s="15" t="inlineStr"/>
+      <c r="O9" s="15" t="inlineStr"/>
+      <c r="P9" s="15" t="n">
+        <v>1161</v>
+      </c>
+      <c r="Q9" s="15" t="inlineStr">
+        <is>
+          <t>submitted</t>
+        </is>
+      </c>
+      <c r="R9" s="15" t="inlineStr"/>
+      <c r="S9" s="15" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="O9" s="15" t="inlineStr"/>
-      <c r="P9" s="15" t="inlineStr">
-        <is>
-          <t>not_affected</t>
-        </is>
-      </c>
-      <c r="Q9" s="15" t="inlineStr"/>
-      <c r="R9" s="15" t="inlineStr"/>
-      <c r="S9" s="15" t="inlineStr"/>
       <c r="T9" s="15" t="inlineStr"/>
       <c r="U9" s="15" t="inlineStr">
         <is>
+          <t>not_affected</t>
+        </is>
+      </c>
+      <c r="V9" s="15" t="inlineStr"/>
+      <c r="W9" s="15" t="inlineStr"/>
+      <c r="X9" s="15" t="inlineStr"/>
+      <c r="Y9" s="15" t="inlineStr"/>
+      <c r="Z9" s="15" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
@@ -1960,12 +2248,12 @@
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>2024-01-28</t>
+          <t>2024-10-21</t>
         </is>
       </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
-          <t>Vikram Trivedi</t>
+          <t>Rahul Grover</t>
         </is>
       </c>
       <c r="H10" s="14" t="inlineStr">
@@ -1975,44 +2263,61 @@
       </c>
       <c r="I10" s="14" t="inlineStr">
         <is>
-          <t>Bengaluru, KA</t>
+          <t>Kolkata, WB</t>
         </is>
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>2024-02-15</t>
-        </is>
-      </c>
-      <c r="K10" s="14" t="n">
-        <v>29640</v>
+          <t>2024-11-09</t>
+        </is>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
       </c>
       <c r="L10" s="14" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="M10" s="14" t="inlineStr">
+        <is>
+          <t>no_answer</t>
+        </is>
+      </c>
+      <c r="N10" s="14" t="inlineStr"/>
+      <c r="O10" s="14" t="inlineStr"/>
+      <c r="P10" s="14" t="n">
+        <v>17178</v>
+      </c>
+      <c r="Q10" s="14" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M10" s="14" t="inlineStr">
-        <is>
-          <t>KA-03-HO-1006</t>
-        </is>
-      </c>
-      <c r="N10" s="14" t="inlineStr">
+      <c r="R10" s="14" t="inlineStr">
+        <is>
+          <t>WB-02-XU-3780</t>
+        </is>
+      </c>
+      <c r="S10" s="14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="O10" s="14" t="inlineStr"/>
-      <c r="P10" s="14" t="inlineStr">
-        <is>
-          <t>not_affected</t>
-        </is>
-      </c>
-      <c r="Q10" s="14" t="inlineStr"/>
-      <c r="R10" s="14" t="inlineStr"/>
-      <c r="S10" s="14" t="inlineStr"/>
       <c r="T10" s="14" t="inlineStr"/>
       <c r="U10" s="14" t="inlineStr">
         <is>
+          <t>not_affected</t>
+        </is>
+      </c>
+      <c r="V10" s="14" t="inlineStr"/>
+      <c r="W10" s="14" t="inlineStr"/>
+      <c r="X10" s="14" t="inlineStr"/>
+      <c r="Y10" s="14" t="inlineStr"/>
+      <c r="Z10" s="14" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
@@ -2045,12 +2350,12 @@
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>2024-03-13</t>
+          <t>2024-04-26</t>
         </is>
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>Ananya Patil</t>
+          <t>Amit Singh</t>
         </is>
       </c>
       <c r="H11" s="15" t="inlineStr">
@@ -2060,55 +2365,80 @@
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>Bengaluru, KA</t>
+          <t>Mumbai, MH</t>
         </is>
       </c>
       <c r="J11" s="15" t="inlineStr">
         <is>
-          <t>2024-04-03</t>
-        </is>
-      </c>
-      <c r="K11" s="15" t="n">
-        <v>31436</v>
+          <t>2024-05-10</t>
+        </is>
+      </c>
+      <c r="K11" s="15" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
       </c>
       <c r="L11" s="15" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="M11" s="15" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="N11" s="15" t="inlineStr">
+        <is>
+          <t>BATTERY_RECALL</t>
+        </is>
+      </c>
+      <c r="O11" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="P11" s="15" t="n">
+        <v>21000</v>
+      </c>
+      <c r="Q11" s="15" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M11" s="15" t="inlineStr">
-        <is>
-          <t>KA-03-NQ-6491</t>
-        </is>
-      </c>
-      <c r="N11" s="15" t="inlineStr">
+      <c r="R11" s="15" t="inlineStr">
+        <is>
+          <t>MH-02-ZP-2193</t>
+        </is>
+      </c>
+      <c r="S11" s="15" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="O11" s="15" t="inlineStr">
+      <c r="T11" s="15" t="inlineStr">
         <is>
           <t>BC-2024-001</t>
         </is>
       </c>
-      <c r="P11" s="15" t="inlineStr">
+      <c r="U11" s="15" t="inlineStr">
         <is>
           <t>in_progress</t>
         </is>
       </c>
-      <c r="Q11" s="15" t="inlineStr">
+      <c r="V11" s="15" t="inlineStr">
         <is>
           <t>BP-LFP-96010</t>
         </is>
       </c>
-      <c r="R11" s="15" t="inlineStr"/>
-      <c r="S11" s="15" t="inlineStr"/>
-      <c r="T11" s="15" t="inlineStr">
-        <is>
-          <t>Vikram Singh</t>
-        </is>
-      </c>
-      <c r="U11" s="15" t="inlineStr">
+      <c r="W11" s="15" t="inlineStr"/>
+      <c r="X11" s="15" t="inlineStr"/>
+      <c r="Y11" s="15" t="inlineStr">
+        <is>
+          <t>Amit Yadav</t>
+        </is>
+      </c>
+      <c r="Z11" s="15" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2142,12 +2472,12 @@
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>2025-07-21</t>
+          <t>2023-01-12</t>
         </is>
       </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
-          <t>Prisha Choudhury</t>
+          <t>Riya Sharma</t>
         </is>
       </c>
       <c r="H12" s="14" t="inlineStr">
@@ -2157,44 +2487,69 @@
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
-          <t>Pune, MH</t>
+          <t>Kolkata, WB</t>
         </is>
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>2025-08-08</t>
-        </is>
-      </c>
-      <c r="K12" s="14" t="n">
-        <v>14268</v>
+          <t>2023-01-20</t>
+        </is>
+      </c>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>2025-01-19</t>
+        </is>
       </c>
       <c r="L12" s="14" t="inlineStr">
         <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="M12" s="14" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="N12" s="14" t="inlineStr">
+        <is>
+          <t>BMS_CELL_IMBALANCE</t>
+        </is>
+      </c>
+      <c r="O12" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="P12" s="14" t="n">
+        <v>33540</v>
+      </c>
+      <c r="Q12" s="14" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M12" s="14" t="inlineStr">
-        <is>
-          <t>MH-12-KD-1090</t>
-        </is>
-      </c>
-      <c r="N12" s="14" t="inlineStr">
+      <c r="R12" s="14" t="inlineStr">
+        <is>
+          <t>WB-02-OX-2988</t>
+        </is>
+      </c>
+      <c r="S12" s="14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="O12" s="14" t="inlineStr"/>
-      <c r="P12" s="14" t="inlineStr">
-        <is>
-          <t>not_affected</t>
-        </is>
-      </c>
-      <c r="Q12" s="14" t="inlineStr"/>
-      <c r="R12" s="14" t="inlineStr"/>
-      <c r="S12" s="14" t="inlineStr"/>
       <c r="T12" s="14" t="inlineStr"/>
       <c r="U12" s="14" t="inlineStr">
         <is>
+          <t>not_affected</t>
+        </is>
+      </c>
+      <c r="V12" s="14" t="inlineStr"/>
+      <c r="W12" s="14" t="inlineStr"/>
+      <c r="X12" s="14" t="inlineStr"/>
+      <c r="Y12" s="14" t="inlineStr"/>
+      <c r="Z12" s="14" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
@@ -2227,12 +2582,12 @@
       </c>
       <c r="F13" s="15" t="inlineStr">
         <is>
-          <t>2024-05-25</t>
+          <t>2025-05-23</t>
         </is>
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>Riya Pillai</t>
+          <t>Ishaan Mehta</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
@@ -2242,44 +2597,61 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>Bengaluru, KA</t>
+          <t>Jaipur, RJ</t>
         </is>
       </c>
       <c r="J13" s="15" t="inlineStr">
         <is>
-          <t>2024-06-02</t>
-        </is>
-      </c>
-      <c r="K13" s="15" t="n">
-        <v>28809</v>
+          <t>2025-06-14</t>
+        </is>
+      </c>
+      <c r="K13" s="15" t="inlineStr">
+        <is>
+          <t>2027-06-14</t>
+        </is>
       </c>
       <c r="L13" s="15" t="inlineStr">
         <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="M13" s="15" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="N13" s="15" t="inlineStr"/>
+      <c r="O13" s="15" t="inlineStr"/>
+      <c r="P13" s="15" t="n">
+        <v>15204</v>
+      </c>
+      <c r="Q13" s="15" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M13" s="15" t="inlineStr">
-        <is>
-          <t>KA-03-NO-6198</t>
-        </is>
-      </c>
-      <c r="N13" s="15" t="inlineStr">
+      <c r="R13" s="15" t="inlineStr">
+        <is>
+          <t>RJ-14-GQ-9540</t>
+        </is>
+      </c>
+      <c r="S13" s="15" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="O13" s="15" t="inlineStr"/>
-      <c r="P13" s="15" t="inlineStr">
-        <is>
-          <t>not_affected</t>
-        </is>
-      </c>
-      <c r="Q13" s="15" t="inlineStr"/>
-      <c r="R13" s="15" t="inlineStr"/>
-      <c r="S13" s="15" t="inlineStr"/>
       <c r="T13" s="15" t="inlineStr"/>
       <c r="U13" s="15" t="inlineStr">
         <is>
+          <t>not_affected</t>
+        </is>
+      </c>
+      <c r="V13" s="15" t="inlineStr"/>
+      <c r="W13" s="15" t="inlineStr"/>
+      <c r="X13" s="15" t="inlineStr"/>
+      <c r="Y13" s="15" t="inlineStr"/>
+      <c r="Z13" s="15" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
@@ -2312,12 +2684,12 @@
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>2024-05-21</t>
+          <t>2024-11-18</t>
         </is>
       </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
-          <t>Sanjay Bose</t>
+          <t>Arjun Yadav</t>
         </is>
       </c>
       <c r="H14" s="14" t="inlineStr">
@@ -2327,63 +2699,80 @@
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
-          <t>Kolkata, WB</t>
+          <t>Bengaluru, KA</t>
         </is>
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>2024-06-15</t>
-        </is>
-      </c>
-      <c r="K14" s="14" t="n">
-        <v>22958</v>
+          <t>2024-12-03</t>
+        </is>
+      </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
       </c>
       <c r="L14" s="14" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="M14" s="14" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="N14" s="14" t="inlineStr"/>
+      <c r="O14" s="14" t="inlineStr"/>
+      <c r="P14" s="14" t="n">
+        <v>15561</v>
+      </c>
+      <c r="Q14" s="14" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M14" s="14" t="inlineStr">
-        <is>
-          <t>WB-02-GL-5681</t>
-        </is>
-      </c>
-      <c r="N14" s="14" t="inlineStr">
+      <c r="R14" s="14" t="inlineStr">
+        <is>
+          <t>KA-03-SS-2052</t>
+        </is>
+      </c>
+      <c r="S14" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="O14" s="14" t="inlineStr">
+      <c r="T14" s="14" t="inlineStr">
         <is>
           <t>BC-2024-001</t>
         </is>
       </c>
-      <c r="P14" s="14" t="inlineStr">
+      <c r="U14" s="14" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="Q14" s="14" t="inlineStr">
+      <c r="V14" s="14" t="inlineStr">
         <is>
           <t>BP-LFP-96013</t>
         </is>
       </c>
-      <c r="R14" s="14" t="inlineStr">
+      <c r="W14" s="14" t="inlineStr">
         <is>
           <t>BP-LFP-96013-R</t>
         </is>
       </c>
-      <c r="S14" s="14" t="inlineStr">
-        <is>
-          <t>2024-12-31</t>
-        </is>
-      </c>
-      <c r="T14" s="14" t="inlineStr">
-        <is>
-          <t>Vikram Singh</t>
-        </is>
-      </c>
-      <c r="U14" s="14" t="inlineStr">
+      <c r="X14" s="14" t="inlineStr">
+        <is>
+          <t>2025-09-18</t>
+        </is>
+      </c>
+      <c r="Y14" s="14" t="inlineStr">
+        <is>
+          <t>Manoj Sharma</t>
+        </is>
+      </c>
+      <c r="Z14" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -2417,12 +2806,12 @@
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>2025-04-29</t>
+          <t>2023-02-10</t>
         </is>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>Riya Patel</t>
+          <t>Aryan Mehta</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
@@ -2432,51 +2821,68 @@
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>Kolkata, WB</t>
+          <t>Chennai, TN</t>
         </is>
       </c>
       <c r="J15" s="15" t="inlineStr">
         <is>
-          <t>2025-05-17</t>
-        </is>
-      </c>
-      <c r="K15" s="15" t="n">
-        <v>14070</v>
+          <t>2023-03-05</t>
+        </is>
+      </c>
+      <c r="K15" s="15" t="inlineStr">
+        <is>
+          <t>2025-03-04</t>
+        </is>
       </c>
       <c r="L15" s="15" t="inlineStr">
         <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="M15" s="15" t="inlineStr">
+        <is>
+          <t>no_answer</t>
+        </is>
+      </c>
+      <c r="N15" s="15" t="inlineStr"/>
+      <c r="O15" s="15" t="inlineStr"/>
+      <c r="P15" s="15" t="n">
+        <v>25452</v>
+      </c>
+      <c r="Q15" s="15" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M15" s="15" t="inlineStr">
-        <is>
-          <t>WB-02-BV-7381</t>
-        </is>
-      </c>
-      <c r="N15" s="15" t="inlineStr">
+      <c r="R15" s="15" t="inlineStr">
+        <is>
+          <t>TN-09-KX-7865</t>
+        </is>
+      </c>
+      <c r="S15" s="15" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="O15" s="15" t="inlineStr">
+      <c r="T15" s="15" t="inlineStr">
         <is>
           <t>BC-2024-001</t>
         </is>
       </c>
-      <c r="P15" s="15" t="inlineStr">
+      <c r="U15" s="15" t="inlineStr">
         <is>
           <t>pending</t>
         </is>
       </c>
-      <c r="Q15" s="15" t="inlineStr">
+      <c r="V15" s="15" t="inlineStr">
         <is>
           <t>BP-LFP-96014</t>
         </is>
       </c>
-      <c r="R15" s="15" t="inlineStr"/>
-      <c r="S15" s="15" t="inlineStr"/>
-      <c r="T15" s="15" t="inlineStr"/>
-      <c r="U15" s="15" t="inlineStr">
+      <c r="W15" s="15" t="inlineStr"/>
+      <c r="X15" s="15" t="inlineStr"/>
+      <c r="Y15" s="15" t="inlineStr"/>
+      <c r="Z15" s="15" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -2510,12 +2916,12 @@
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>2025-03-09</t>
+          <t>2025-03-07</t>
         </is>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
-          <t>Alok Chatterjee</t>
+          <t>Rohit Rao</t>
         </is>
       </c>
       <c r="H16" s="14" t="inlineStr">
@@ -2525,63 +2931,80 @@
       </c>
       <c r="I16" s="14" t="inlineStr">
         <is>
-          <t>Kolkata, WB</t>
+          <t>Jaipur, RJ</t>
         </is>
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>2025-03-27</t>
-        </is>
-      </c>
-      <c r="K16" s="14" t="n">
-        <v>19567</v>
+          <t>2025-03-22</t>
+        </is>
+      </c>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>2027-03-22</t>
+        </is>
       </c>
       <c r="L16" s="14" t="inlineStr">
         <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="M16" s="14" t="inlineStr">
+        <is>
+          <t>message_sent</t>
+        </is>
+      </c>
+      <c r="N16" s="14" t="inlineStr"/>
+      <c r="O16" s="14" t="inlineStr"/>
+      <c r="P16" s="14" t="n">
+        <v>13073</v>
+      </c>
+      <c r="Q16" s="14" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M16" s="14" t="inlineStr">
-        <is>
-          <t>WB-02-FF-8140</t>
-        </is>
-      </c>
-      <c r="N16" s="14" t="inlineStr">
+      <c r="R16" s="14" t="inlineStr">
+        <is>
+          <t>RJ-14-NX-1444</t>
+        </is>
+      </c>
+      <c r="S16" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="O16" s="14" t="inlineStr">
+      <c r="T16" s="14" t="inlineStr">
         <is>
           <t>BC-2024-001</t>
         </is>
       </c>
-      <c r="P16" s="14" t="inlineStr">
+      <c r="U16" s="14" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="Q16" s="14" t="inlineStr">
+      <c r="V16" s="14" t="inlineStr">
         <is>
           <t>BP-NMC-72015</t>
         </is>
       </c>
-      <c r="R16" s="14" t="inlineStr">
+      <c r="W16" s="14" t="inlineStr">
         <is>
           <t>BP-NMC-72015-R</t>
         </is>
       </c>
-      <c r="S16" s="14" t="inlineStr">
-        <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="T16" s="14" t="inlineStr">
+      <c r="X16" s="14" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="Y16" s="14" t="inlineStr">
         <is>
           <t>Rajesh Kumar</t>
         </is>
       </c>
-      <c r="U16" s="14" t="inlineStr">
+      <c r="Z16" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -2615,12 +3038,12 @@
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2025-07-20</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>Raj Trivedi</t>
+          <t>Ishaan Sen</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -2635,58 +3058,75 @@
       </c>
       <c r="J17" s="15" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="K17" s="15" t="n">
-        <v>627</v>
+          <t>2025-08-04</t>
+        </is>
+      </c>
+      <c r="K17" s="15" t="inlineStr">
+        <is>
+          <t>2027-08-04</t>
+        </is>
       </c>
       <c r="L17" s="15" t="inlineStr">
         <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="M17" s="15" t="inlineStr">
+        <is>
+          <t>no_answer</t>
+        </is>
+      </c>
+      <c r="N17" s="15" t="inlineStr"/>
+      <c r="O17" s="15" t="inlineStr"/>
+      <c r="P17" s="15" t="n">
+        <v>11492</v>
+      </c>
+      <c r="Q17" s="15" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M17" s="15" t="inlineStr">
-        <is>
-          <t>GJ-01-CL-8564</t>
-        </is>
-      </c>
-      <c r="N17" s="15" t="inlineStr">
+      <c r="R17" s="15" t="inlineStr">
+        <is>
+          <t>GJ-01-CA-9837</t>
+        </is>
+      </c>
+      <c r="S17" s="15" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="O17" s="15" t="inlineStr">
+      <c r="T17" s="15" t="inlineStr">
         <is>
           <t>BC-2024-001</t>
         </is>
       </c>
-      <c r="P17" s="15" t="inlineStr">
+      <c r="U17" s="15" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="Q17" s="15" t="inlineStr">
+      <c r="V17" s="15" t="inlineStr">
         <is>
           <t>BP-NMC-72016</t>
         </is>
       </c>
-      <c r="R17" s="15" t="inlineStr">
+      <c r="W17" s="15" t="inlineStr">
         <is>
           <t>BP-NMC-72016-R</t>
         </is>
       </c>
-      <c r="S17" s="15" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="T17" s="15" t="inlineStr">
-        <is>
-          <t>Arjun Patel</t>
-        </is>
-      </c>
-      <c r="U17" s="15" t="inlineStr">
+      <c r="X17" s="15" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="Y17" s="15" t="inlineStr">
+        <is>
+          <t>Vikram Singh</t>
+        </is>
+      </c>
+      <c r="Z17" s="15" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -2720,12 +3160,12 @@
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>2025-02-15</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
-          <t>Diya Kumar</t>
+          <t>Vijay Nair</t>
         </is>
       </c>
       <c r="H18" s="14" t="inlineStr">
@@ -2735,63 +3175,76 @@
       </c>
       <c r="I18" s="14" t="inlineStr">
         <is>
-          <t>Jaipur, RJ</t>
+          <t>Delhi, DL</t>
         </is>
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>2025-03-02</t>
-        </is>
-      </c>
-      <c r="K18" s="14" t="n">
-        <v>14688</v>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>2028-07-04</t>
+        </is>
       </c>
       <c r="L18" s="14" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="M18" s="14" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="N18" s="14" t="inlineStr"/>
+      <c r="O18" s="14" t="inlineStr"/>
+      <c r="P18" s="14" t="n">
+        <v>1084</v>
+      </c>
+      <c r="Q18" s="14" t="inlineStr">
+        <is>
+          <t>delivered</t>
+        </is>
+      </c>
+      <c r="R18" s="14" t="inlineStr"/>
+      <c r="S18" s="14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="T18" s="14" t="inlineStr">
+        <is>
+          <t>BC-2024-001</t>
+        </is>
+      </c>
+      <c r="U18" s="14" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M18" s="14" t="inlineStr">
-        <is>
-          <t>RJ-14-TJ-7906</t>
-        </is>
-      </c>
-      <c r="N18" s="14" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="O18" s="14" t="inlineStr">
-        <is>
-          <t>BC-2024-001</t>
-        </is>
-      </c>
-      <c r="P18" s="14" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="Q18" s="14" t="inlineStr">
+      <c r="V18" s="14" t="inlineStr">
         <is>
           <t>BP-LFP-96017</t>
         </is>
       </c>
-      <c r="R18" s="14" t="inlineStr">
+      <c r="W18" s="14" t="inlineStr">
         <is>
           <t>BP-LFP-96017-R</t>
         </is>
       </c>
-      <c r="S18" s="14" t="inlineStr">
-        <is>
-          <t>2025-07-05</t>
-        </is>
-      </c>
-      <c r="T18" s="14" t="inlineStr">
-        <is>
-          <t>Amit Yadav</t>
-        </is>
-      </c>
-      <c r="U18" s="14" t="inlineStr">
+      <c r="X18" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="Y18" s="14" t="inlineStr">
+        <is>
+          <t>Rajesh Kumar</t>
+        </is>
+      </c>
+      <c r="Z18" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -2825,12 +3278,12 @@
       </c>
       <c r="F19" s="15" t="inlineStr">
         <is>
-          <t>2023-03-24</t>
+          <t>2024-09-29</t>
         </is>
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>Priya Rao</t>
+          <t>Prisha Yadav</t>
         </is>
       </c>
       <c r="H19" s="15" t="inlineStr">
@@ -2840,60 +3293,80 @@
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
-          <t>Pune, MH</t>
+          <t>Lucknow, UP</t>
         </is>
       </c>
       <c r="J19" s="15" t="inlineStr">
         <is>
-          <t>2023-03-29</t>
-        </is>
-      </c>
-      <c r="K19" s="15" t="n">
-        <v>34973</v>
+          <t>2024-10-07</t>
+        </is>
+      </c>
+      <c r="K19" s="15" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
       </c>
       <c r="L19" s="15" t="inlineStr">
         <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="M19" s="15" t="inlineStr">
+        <is>
+          <t>connected</t>
+        </is>
+      </c>
+      <c r="N19" s="15" t="inlineStr"/>
+      <c r="O19" s="15" t="inlineStr"/>
+      <c r="P19" s="15" t="n">
+        <v>21137</v>
+      </c>
+      <c r="Q19" s="15" t="inlineStr">
+        <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="M19" s="15" t="inlineStr">
-        <is>
-          <t>MH-12-DD-2874</t>
-        </is>
-      </c>
-      <c r="N19" s="15" t="inlineStr">
+      <c r="R19" s="15" t="inlineStr">
+        <is>
+          <t>UP-32-YF-4978</t>
+        </is>
+      </c>
+      <c r="S19" s="15" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="O19" s="15" t="inlineStr"/>
-      <c r="P19" s="15" t="inlineStr">
-        <is>
-          <t>not_affected</t>
-        </is>
-      </c>
-      <c r="Q19" s="15" t="inlineStr"/>
-      <c r="R19" s="15" t="inlineStr"/>
-      <c r="S19" s="15" t="inlineStr"/>
       <c r="T19" s="15" t="inlineStr"/>
       <c r="U19" s="15" t="inlineStr">
         <is>
+          <t>not_affected</t>
+        </is>
+      </c>
+      <c r="V19" s="15" t="inlineStr"/>
+      <c r="W19" s="15" t="inlineStr"/>
+      <c r="X19" s="15" t="inlineStr"/>
+      <c r="Y19" s="15" t="inlineStr"/>
+      <c r="Z19" s="15" t="inlineStr">
+        <is>
           <t>FALSE</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="B2:B300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Model" error="Your entry is not in the list of allowed vehicle models (CT2, CO1)" promptTitle="Select EV Model" prompt="Please select CT2 or CO1" type="list">
       <formula1>"CT2,CO1"</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Registration Status" error="Must choose delivered, documents_pending, submitted, or completed" promptTitle="Select Status" prompt="Select registration stage" type="list">
+    <dataValidation sqref="Q2:Q300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Registration Status" error="Must choose delivered, documents_pending, submitted, or completed" promptTitle="Select Status" prompt="Select registration stage" type="list">
       <formula1>"delivered,documents_pending,submitted,completed"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Upgrade Status" error="Must choose not_affected, pending, in_progress, or completed" type="list">
+    <dataValidation sqref="M2:M300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Contact Outcome" error="Must choose connected, no_answer, or message_sent" type="list">
+      <formula1>"connected,no_answer,message_sent"</formula1>
+    </dataValidation>
+    <dataValidation sqref="U2:U300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Upgrade Status" error="Must choose not_affected, pending, in_progress, or completed" type="list">
       <formula1>"not_affected,pending,in_progress,completed"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N300 U2:U300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Boolean Value" error="Must enter TRUE or FALSE" type="list">
+    <dataValidation sqref="S2:S300 Z2:Z300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Boolean Value" error="Must enter TRUE or FALSE" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>